<commit_message>
Add ReportTutor And Add RequestWithdraw
</commit_message>
<xml_diff>
--- a/ExcelProject/Login.xlsx
+++ b/ExcelProject/Login.xlsx
@@ -40,7 +40,7 @@
     <t>Revise</t>
   </si>
   <si>
-    <t>Y</t>
+    <t>N</t>
   </si>
   <si>
     <t>TC3:01</t>
@@ -648,7 +648,7 @@
     <col min="8" max="8" style="6" width="14.147857142857141" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="27.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="27">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -674,7 +674,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="21.75">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -698,7 +698,7 @@
       </c>
       <c r="H2" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21.75">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -722,7 +722,7 @@
       </c>
       <c r="H3" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="21.75">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
@@ -746,7 +746,7 @@
       </c>
       <c r="H4" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21.75">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
@@ -770,7 +770,7 @@
       </c>
       <c r="H5" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21.75">
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
@@ -794,7 +794,7 @@
       </c>
       <c r="H6" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21.75">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
@@ -818,7 +818,7 @@
       </c>
       <c r="H7" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="21.75">
       <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
@@ -842,7 +842,7 @@
       </c>
       <c r="H8" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="21.75">
       <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
@@ -864,7 +864,7 @@
       </c>
       <c r="H9" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="21.75">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
@@ -888,7 +888,7 @@
       </c>
       <c r="H10" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="21.75">
       <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
@@ -912,7 +912,7 @@
       </c>
       <c r="H11" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="21.75">
       <c r="A12" s="3" t="s">
         <v>8</v>
       </c>
@@ -936,7 +936,7 @@
       </c>
       <c r="H12" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="21.75">
       <c r="A13" s="3" t="s">
         <v>8</v>
       </c>
@@ -960,7 +960,7 @@
       </c>
       <c r="H13" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="21.75">
       <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
@@ -984,7 +984,7 @@
       </c>
       <c r="H14" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="21.75">
       <c r="A15" s="3" t="s">
         <v>8</v>
       </c>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H15" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="21.75">
       <c r="A16" s="3" t="s">
         <v>8</v>
       </c>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H16" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="21.75">
       <c r="A17" s="3" t="s">
         <v>8</v>
       </c>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="H17" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="21.75">
       <c r="A18" s="3" t="s">
         <v>8</v>
       </c>

</xml_diff>